<commit_message>
Updated 6 feature file may6
</commit_message>
<xml_diff>
--- a/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
+++ b/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="39">
   <si>
     <t>TC ID</t>
   </si>
@@ -110,10 +110,13 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>22 Apr 2026</t>
-  </si>
-  <si>
-    <t>REQ-619</t>
+    <t>4 May 2026</t>
+  </si>
+  <si>
+    <t>1 May 2026</t>
+  </si>
+  <si>
+    <t>REQ-621</t>
   </si>
   <si>
     <t>TC002</t>
@@ -137,10 +140,10 @@
     <t>${TC001.Odometer}</t>
   </si>
   <si>
-    <t>5016</t>
-  </si>
-  <si>
-    <t>REQ-621</t>
+    <t>12300</t>
+  </si>
+  <si>
+    <t>REQ-651</t>
   </si>
 </sst>
 </file>
@@ -810,10 +813,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -828,7 +831,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1253,15 +1256,15 @@
         <v>23</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="6">
         <f>C2+1</f>
-        <v>5017</v>
+        <v>12301</v>
       </c>
       <c r="E2" s="6">
         <f>D2</f>
-        <v>5017</v>
+        <v>12301</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>24</v>
@@ -1306,30 +1309,30 @@
         <v>27</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="V2" s="8" t="str">
+        <v>38</v>
+      </c>
+      <c r="V2" s="7" t="str">
         <f>TEXT(E2,"#,##0")&amp;" km"</f>
-        <v>5,017 km</v>
-      </c>
-      <c r="W2" s="8"/>
+        <v>12,301 km</v>
+      </c>
+      <c r="W2" s="7"/>
     </row>
     <row r="3" s="2" customFormat="1" ht="55.2" spans="1:23">
       <c r="A3" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>24</v>
@@ -1371,23 +1374,23 @@
         <v>26</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W3" s="4"/>
     </row>
-    <row r="5" spans="5:5">
-      <c r="E5" s="7"/>
+    <row r="5" spans="1:23">
+      <c r="E5" s="8"/>
     </row>
-    <row r="10" spans="21:21">
+    <row r="10" spans="1:23">
       <c r="U10" s="9"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ExcelWriter updates and new methods to handle labels
</commit_message>
<xml_diff>
--- a/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
+++ b/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
   <si>
     <t>TC ID</t>
   </si>
@@ -95,12 +95,54 @@
     <t>Odometer</t>
   </si>
   <si>
+    <t>Driver Salutation</t>
+  </si>
+  <si>
+    <t>Driver First Name</t>
+  </si>
+  <si>
+    <t>Driver Last Name</t>
+  </si>
+  <si>
+    <t>Driver Name</t>
+  </si>
+  <si>
+    <t>Driver Date of Birth</t>
+  </si>
+  <si>
+    <t>Driver Mobile Phone</t>
+  </si>
+  <si>
+    <t>Driver Email</t>
+  </si>
+  <si>
+    <t>Driver Your Residential Address</t>
+  </si>
+  <si>
+    <t>Driver Employer Name</t>
+  </si>
+  <si>
+    <t>Vehicle</t>
+  </si>
+  <si>
+    <t>Vehicle number</t>
+  </si>
+  <si>
+    <t>Vehicle name</t>
+  </si>
+  <si>
+    <t>Lease End Date</t>
+  </si>
+  <si>
     <t>TC001</t>
   </si>
   <si>
     <t>Reimbursement Claim</t>
   </si>
   <si>
+    <t>12308</t>
+  </si>
+  <si>
     <t>Fuel</t>
   </si>
   <si>
@@ -110,13 +152,28 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>4 May 2026</t>
-  </si>
-  <si>
-    <t>1 May 2026</t>
-  </si>
-  <si>
-    <t>REQ-621</t>
+    <t>7 May 2026</t>
+  </si>
+  <si>
+    <t>REQ-669</t>
+  </si>
+  <si>
+    <t>Mr</t>
+  </si>
+  <si>
+    <t>Toshihiko</t>
+  </si>
+  <si>
+    <t>Inafune</t>
+  </si>
+  <si>
+    <t>FTV21M</t>
+  </si>
+  <si>
+    <t>MAZDA CX-5</t>
+  </si>
+  <si>
+    <t>30 Aug 2029</t>
   </si>
   <si>
     <t>TC002</t>
@@ -128,6 +185,15 @@
     <t>${TC001.New Odometer}</t>
   </si>
   <si>
+    <t>${TC001.Claim Type}</t>
+  </si>
+  <si>
+    <t>${TC001.Amount ($)}</t>
+  </si>
+  <si>
+    <t>${TC001.Proof of Payment}</t>
+  </si>
+  <si>
     <t>${TC001.Reading Date}</t>
   </si>
   <si>
@@ -140,10 +206,34 @@
     <t>${TC001.Odometer}</t>
   </si>
   <si>
-    <t>12300</t>
-  </si>
-  <si>
-    <t>REQ-651</t>
+    <t>${TC001.Driver Salutation}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver First Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Last Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Date of Birth}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Mobile Phone}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Email}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Your Residential Address}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Employer Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle}</t>
   </si>
 </sst>
 </file>
@@ -1157,29 +1247,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:W10"/>
+  <dimension ref="A1:AI10"/>
   <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="8.55833333333333"/>
-    <col min="2" max="2" customWidth="true" width="20.7"/>
-    <col min="3" max="4" customWidth="true" width="24.3333333333333"/>
-    <col min="5" max="5" customWidth="true" width="27.3333333333333"/>
-    <col min="6" max="6" customWidth="true" width="16.775"/>
-    <col min="7" max="7" customWidth="true" width="15.3333333333333"/>
-    <col min="8" max="8" customWidth="true" width="21.775"/>
-    <col min="9" max="9" customWidth="true" width="18.6666666666667"/>
-    <col min="10" max="10" customWidth="true" width="23.775"/>
-    <col min="11" max="11" customWidth="true" width="17.225"/>
-    <col min="12" max="12" customWidth="true" width="19.8916666666667"/>
-    <col min="13" max="13" customWidth="true" width="20.6666666666667"/>
-    <col min="14" max="14" customWidth="true" width="17.5583333333333"/>
-    <col min="15" max="15" customWidth="true" width="14.6666666666667"/>
-    <col min="16" max="16" customWidth="true" width="19.3333333333333"/>
-    <col min="17" max="17" customWidth="true" width="18.4416666666667"/>
-    <col min="18" max="23" customWidth="true" width="19.1083333333333"/>
+    <col min="1" max="1" width="8.55833333333333" customWidth="1"/>
+    <col min="2" max="2" width="20.7" customWidth="1"/>
+    <col min="3" max="4" width="24.3333333333333" customWidth="1"/>
+    <col min="5" max="5" width="27.3333333333333" customWidth="1"/>
+    <col min="6" max="6" width="16.775" customWidth="1"/>
+    <col min="7" max="7" width="15.3333333333333" customWidth="1"/>
+    <col min="8" max="8" width="21.775" customWidth="1"/>
+    <col min="9" max="9" width="18.6666666666667" customWidth="1"/>
+    <col min="10" max="10" width="23.775" customWidth="1"/>
+    <col min="11" max="11" width="17.225" customWidth="1"/>
+    <col min="12" max="12" width="19.8916666666667" customWidth="1"/>
+    <col min="13" max="13" width="20.6666666666667" customWidth="1"/>
+    <col min="14" max="14" width="17.5583333333333" customWidth="1"/>
+    <col min="15" max="15" width="14.6666666666667" customWidth="1"/>
+    <col min="16" max="16" width="19.3333333333333" customWidth="1"/>
+    <col min="17" max="17" width="18.4416666666667" customWidth="1"/>
+    <col min="18" max="32" width="19.1083333333333" customWidth="1"/>
+    <col min="33" max="33" width="15.1" customWidth="1"/>
+    <col min="34" max="34" width="12.8" customWidth="1"/>
+    <col min="35" max="35" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="27.6" spans="1:23">
+    <row r="1" s="1" customFormat="1" ht="27.6" spans="1:35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1246,151 +1339,252 @@
       <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3"/>
+      <c r="W1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" s="2" customFormat="1" ht="55.2" spans="1:23">
+    <row r="2" s="2" customFormat="1" ht="55.2" spans="1:35">
       <c r="A2" s="4" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D2" s="6">
         <f>C2+1</f>
-        <v>12301</v>
+        <v>12309</v>
       </c>
       <c r="E2" s="6">
         <f>D2</f>
-        <v>12301</v>
+        <v>12309</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="G2" s="4">
         <v>300</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="V2" s="7" t="str">
         <f>TEXT(E2,"#,##0")&amp;" km"</f>
-        <v>12,301 km</v>
-      </c>
-      <c r="W2" s="7"/>
+        <v>12,309 km</v>
+      </c>
+      <c r="W2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" s="7" t="str">
+        <f>_xlfn.CONCAT(X2," ",Y2)</f>
+        <v>Toshihiko Inafune</v>
+      </c>
+      <c r="AA2" s="7"/>
+      <c r="AB2" s="7"/>
+      <c r="AC2" s="7"/>
+      <c r="AD2" s="7"/>
+      <c r="AE2" s="7"/>
+      <c r="AF2" s="7"/>
+      <c r="AG2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI2" s="7" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="3" s="2" customFormat="1" ht="55.2" spans="1:23">
+    <row r="3" s="2" customFormat="1" ht="27.6" spans="1:35">
       <c r="A3" s="4" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="4">
-        <v>300</v>
+        <v>52</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>53</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="W3" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AB3" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AC3" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AH3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI3" s="4"/>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:35">
       <c r="E5" s="8"/>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:35">
       <c r="U10" s="9"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completion of End to End Flow
</commit_message>
<xml_diff>
--- a/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
+++ b/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="TestData" sheetId="14" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="76">
   <si>
     <t>TC ID</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Reimbursement Claim</t>
   </si>
   <si>
-    <t>12308</t>
-  </si>
-  <si>
     <t>Fuel</t>
   </si>
   <si>
@@ -152,10 +149,7 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>7 May 2026</t>
-  </si>
-  <si>
-    <t>REQ-669</t>
+    <t>12 May 2026</t>
   </si>
   <si>
     <t>Mr</t>
@@ -167,6 +161,21 @@
     <t>Inafune</t>
   </si>
   <si>
+    <t>05/06/1995</t>
+  </si>
+  <si>
+    <t>0469750861</t>
+  </si>
+  <si>
+    <t>inafune@jfcaust.com.au.test</t>
+  </si>
+  <si>
+    <t>Your Residential Address *</t>
+  </si>
+  <si>
+    <t>JFC Australia Co Pty Ltd</t>
+  </si>
+  <si>
     <t>FTV21M</t>
   </si>
   <si>
@@ -234,6 +243,18 @@
   </si>
   <si>
     <t>${TC001.Vehicle}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle number}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle name}</t>
+  </si>
+  <si>
+    <t>${TC001.Lease End Date}</t>
+  </si>
+  <si>
+    <t>12315</t>
   </si>
 </sst>
 </file>
@@ -1250,26 +1271,27 @@
   <dimension ref="A1:AI10"/>
   <sheetFormatPr defaultColWidth="8.89166666666667" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="8.55833333333333" customWidth="1"/>
-    <col min="2" max="2" width="20.7" customWidth="1"/>
-    <col min="3" max="4" width="24.3333333333333" customWidth="1"/>
-    <col min="5" max="5" width="27.3333333333333" customWidth="1"/>
-    <col min="6" max="6" width="16.775" customWidth="1"/>
-    <col min="7" max="7" width="15.3333333333333" customWidth="1"/>
-    <col min="8" max="8" width="21.775" customWidth="1"/>
-    <col min="9" max="9" width="18.6666666666667" customWidth="1"/>
-    <col min="10" max="10" width="23.775" customWidth="1"/>
-    <col min="11" max="11" width="17.225" customWidth="1"/>
-    <col min="12" max="12" width="19.8916666666667" customWidth="1"/>
-    <col min="13" max="13" width="20.6666666666667" customWidth="1"/>
-    <col min="14" max="14" width="17.5583333333333" customWidth="1"/>
-    <col min="15" max="15" width="14.6666666666667" customWidth="1"/>
-    <col min="16" max="16" width="19.3333333333333" customWidth="1"/>
-    <col min="17" max="17" width="18.4416666666667" customWidth="1"/>
-    <col min="18" max="32" width="19.1083333333333" customWidth="1"/>
-    <col min="33" max="33" width="15.1" customWidth="1"/>
-    <col min="34" max="34" width="12.8" customWidth="1"/>
-    <col min="35" max="35" width="15.5" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.55833333333333"/>
+    <col min="2" max="2" customWidth="true" width="20.7"/>
+    <col min="3" max="4" customWidth="true" width="24.3333333333333"/>
+    <col min="5" max="5" customWidth="true" width="27.3333333333333"/>
+    <col min="6" max="6" customWidth="true" width="16.775"/>
+    <col min="7" max="7" customWidth="true" width="15.3333333333333"/>
+    <col min="8" max="8" customWidth="true" width="21.775"/>
+    <col min="9" max="9" customWidth="true" width="18.6666666666667"/>
+    <col min="10" max="10" customWidth="true" width="23.775"/>
+    <col min="11" max="11" customWidth="true" width="17.225"/>
+    <col min="12" max="12" customWidth="true" width="19.8916666666667"/>
+    <col min="13" max="13" customWidth="true" width="20.6666666666667"/>
+    <col min="14" max="14" customWidth="true" width="17.5583333333333"/>
+    <col min="15" max="15" customWidth="true" width="14.6666666666667"/>
+    <col min="16" max="16" customWidth="true" width="19.3333333333333"/>
+    <col min="17" max="17" customWidth="true" width="18.4416666666667"/>
+    <col min="18" max="31" customWidth="true" width="19.1083333333333"/>
+    <col min="32" max="32" customWidth="true" width="27.2"/>
+    <col min="33" max="33" customWidth="true" width="15.1"/>
+    <col min="34" max="34" customWidth="true" width="12.8"/>
+    <col min="35" max="35" customWidth="true" width="15.5"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="27.6" spans="1:35">
@@ -1387,199 +1409,212 @@
         <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <f>C2+1</f>
+        <v>12316.0</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <f>D2</f>
+        <v>12316.0</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="D2" s="6">
-        <f>C2+1</f>
-        <v>12309</v>
-      </c>
-      <c r="E2" s="6">
-        <f>D2</f>
-        <v>12309</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="G2" s="4">
         <v>300</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>42</v>
-      </c>
+      <c r="U2" s="4"/>
       <c r="V2" s="7" t="str">
         <f>TEXT(E2,"#,##0")&amp;" km"</f>
-        <v>12,309 km</v>
+        <v>12,316 km</v>
       </c>
       <c r="W2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y2" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="X2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y2" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="Z2" s="7" t="str">
         <f>_xlfn.CONCAT(X2," ",Y2)</f>
         <v>Toshihiko Inafune</v>
       </c>
-      <c r="AA2" s="7"/>
-      <c r="AB2" s="7"/>
-      <c r="AC2" s="7"/>
-      <c r="AD2" s="7"/>
-      <c r="AE2" s="7"/>
-      <c r="AF2" s="7"/>
+      <c r="AA2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" s="7" t="str">
+        <f>AH2&amp;" - "&amp;AG2</f>
+        <v>MAZDA CX-5 - FTV21M</v>
+      </c>
       <c r="AG2" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="AH2" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="AI2" s="7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" s="2" customFormat="1" ht="27.6" spans="1:35">
       <c r="A3" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="W3" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="X3" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Y3" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="Z3" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AA3" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AB3" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AC3" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="AD3" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="AF3" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AG3" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AH3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AI3" s="4"/>
+        <v>73</v>
+      </c>
+      <c r="AI3" s="4" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="5" spans="1:35">
       <c r="E5" s="8"/>
@@ -1589,6 +1624,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flow completed till May 25
</commit_message>
<xml_diff>
--- a/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
+++ b/cucumber-for-appian/src/test/resources/testdata/End2End/01_NovatedApp_End2End.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="83">
   <si>
     <t>TC ID</t>
   </si>
@@ -149,7 +149,85 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>12 May 2026</t>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>${TC001.Last Odometer Reading}</t>
+  </si>
+  <si>
+    <t>${TC001.New Odometer}</t>
+  </si>
+  <si>
+    <t>${TC001.Claim Type}</t>
+  </si>
+  <si>
+    <t>${TC001.Amount ($)}</t>
+  </si>
+  <si>
+    <t>${TC001.Proof of Payment}</t>
+  </si>
+  <si>
+    <t>${TC001.Reading Date}</t>
+  </si>
+  <si>
+    <t>${TC001.Last Reading Date}</t>
+  </si>
+  <si>
+    <t>${TC001.Reference Number}</t>
+  </si>
+  <si>
+    <t>${TC001.Odometer}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Salutation}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver First Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Last Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Date of Birth}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Mobile Phone}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Email}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Your Residential Address}</t>
+  </si>
+  <si>
+    <t>${TC001.Driver Employer Name}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle number}</t>
+  </si>
+  <si>
+    <t>${TC001.Vehicle name}</t>
+  </si>
+  <si>
+    <t>${TC001.Lease End Date}</t>
+  </si>
+  <si>
+    <t>FTV21M</t>
+  </si>
+  <si>
+    <t>MAZDA CX-5</t>
+  </si>
+  <si>
+    <t>30 Aug 2029</t>
+  </si>
+  <si>
+    <t>12316</t>
   </si>
   <si>
     <t>Mr</t>
@@ -176,85 +254,28 @@
     <t>JFC Australia Co Pty Ltd</t>
   </si>
   <si>
-    <t>FTV21M</t>
-  </si>
-  <si>
-    <t>MAZDA CX-5</t>
-  </si>
-  <si>
-    <t>30 Aug 2029</t>
-  </si>
-  <si>
-    <t>TC002</t>
-  </si>
-  <si>
-    <t>${TC001.Last Odometer Reading}</t>
-  </si>
-  <si>
-    <t>${TC001.New Odometer}</t>
-  </si>
-  <si>
-    <t>${TC001.Claim Type}</t>
-  </si>
-  <si>
-    <t>${TC001.Amount ($)}</t>
-  </si>
-  <si>
-    <t>${TC001.Proof of Payment}</t>
-  </si>
-  <si>
-    <t>${TC001.Reading Date}</t>
-  </si>
-  <si>
-    <t>${TC001.Last Reading Date}</t>
-  </si>
-  <si>
-    <t>${TC001.Reference Number}</t>
-  </si>
-  <si>
-    <t>${TC001.Odometer}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Salutation}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver First Name}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Last Name}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Name}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Date of Birth}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Mobile Phone}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Email}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Your Residential Address}</t>
-  </si>
-  <si>
-    <t>${TC001.Driver Employer Name}</t>
-  </si>
-  <si>
-    <t>${TC001.Vehicle}</t>
-  </si>
-  <si>
-    <t>${TC001.Vehicle number}</t>
-  </si>
-  <si>
-    <t>${TC001.Vehicle name}</t>
-  </si>
-  <si>
-    <t>${TC001.Lease End Date}</t>
-  </si>
-  <si>
-    <t>12315</t>
+    <t>19 May 2026</t>
+  </si>
+  <si>
+    <t>REQ-714</t>
+  </si>
+  <si>
+    <t>12317</t>
+  </si>
+  <si>
+    <t>REQ-719</t>
+  </si>
+  <si>
+    <t>12318</t>
+  </si>
+  <si>
+    <t>REQ-722</t>
+  </si>
+  <si>
+    <t>12319</t>
+  </si>
+  <si>
+    <t>REQ-729</t>
   </si>
 </sst>
 </file>
@@ -1409,21 +1430,21 @@
         <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D2" s="6" t="n">
         <f>C2+1</f>
-        <v>12316.0</v>
+        <v>12320.0</v>
       </c>
       <c r="E2" s="6" t="n">
         <f>D2</f>
-        <v>12316.0</v>
+        <v>12320.0</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>37</v>
       </c>
       <c r="G2" s="4">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>38</v>
@@ -1459,161 +1480,163 @@
         <v>39</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="U2" s="4"/>
+        <v>75</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="V2" s="7" t="str">
         <f>TEXT(E2,"#,##0")&amp;" km"</f>
-        <v>12,316 km</v>
+        <v>12,320 km</v>
       </c>
       <c r="W2" s="7" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="Y2" s="7" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="Z2" s="7" t="str">
         <f>_xlfn.CONCAT(X2," ",Y2)</f>
         <v>Toshihiko Inafune</v>
       </c>
       <c r="AA2" s="7" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="AB2" s="7" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="AC2" s="7" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="AD2" s="7" t="s">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="AE2" s="7" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="AF2" s="7" t="str">
         <f>AH2&amp;" - "&amp;AG2</f>
         <v>MAZDA CX-5 - FTV21M</v>
       </c>
       <c r="AG2" s="7" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="AH2" s="7" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="AI2" s="7" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" s="2" customFormat="1" ht="27.6" spans="1:35">
       <c r="A3" s="4" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="AB3" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="AC3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="AD3" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" s="4" t="s">
+      <c r="AE3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="AF3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="AG3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="AH3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="AI3" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="X3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="AA3" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AB3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AD3" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AE3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AF3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AG3" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AH3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AI3" s="4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:35">

</xml_diff>